<commit_message>
publish: push main (9000ab0)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit b373025 (built 2026-10-15 15:22 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 9000ab0 (built 2026-10-15 16:06 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b373025 · built 2026-10-15 15:22 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (232c17d)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 9000ab0 (built 2026-10-15 16:06 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 232c17d (built 2026-10-15 16:51 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 9000ab0 · built 2026-10-15 16:06 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (47e0b89)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 232c17d (built 2026-10-15 16:51 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 47e0b89 (built 2026-10-16 13:14 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 232c17d · built 2026-10-15 16:51 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (1eb4564)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 47e0b89 (built 2026-10-16 13:14 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 1eb4564 (built 2026-10-19 09:56 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 47e0b89 · built 2026-10-16 13:14 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (ae2eabb)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 1eb4564 (built 2026-10-19 09:56 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit ae2eabb (built 2026-10-19 10:13 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 1eb4564 · built 2026-10-19 09:56 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (a02e58b)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit ae2eabb (built 2026-10-19 10:13 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit a02e58b (built 2026-10-19 11:55 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit ae2eabb · built 2026-10-19 10:13 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (70c4cff)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit a02e58b (built 2026-10-19 11:55 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 70c4cff (built 2026-10-19 12:11 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit a02e58b · built 2026-10-19 11:55 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (8353c43)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 70c4cff (built 2026-10-19 12:11 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 8353c43 (built 2026-10-19 13:11 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 70c4cff · built 2026-10-19 12:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (b02b579)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit 8353c43 (built 2026-10-19 13:11 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit b02b579 (built 2026-10-19 17:33 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 8353c43 · built 2026-10-19 13:11 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>

<commit_message>
publish: push main (54cc0be)
</commit_message>
<xml_diff>
--- a/draft/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/draft/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch main · commit b02b579 (built 2026-10-19 17:33 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch main · commit 54cc0be (built 2026-10-19 17:40 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7369,7 +7369,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12350,7 +12350,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14483,7 +14483,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27252,7 +27252,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28562,7 +28562,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29154,7 +29154,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32465,7 +32465,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33647,7 +33647,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35142,7 +35142,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37310,7 +37310,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42583,7 +42583,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -46793,7 +46793,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit b02b579 · built 2026-10-19 17:33 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch main · commit 54cc0be · built 2026-10-19 17:40 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>